<commit_message>
feat: evolução arquitetural - SQS Workers, S3 direto, EventBridge, versionamento
Migração do Brand Watchdog para arquitetura distribuída:
- SQSPublisher + SQSConsumer para paralelização via fila
- WorkerMain (ECS Fargate) com timeout 120s e visibility renewal
- ScreenshotStore refatorado para upload S3 direto (multipart >5MB)
- EventPublisher + EventNotificationHandler (dedup + DLQ)
- CycleConsolidator com polling 30s e timeout 60min
- MonitoringCoordinator refatorado (não processa sites diretamente)
- RuleSetVersionCalculator (SHA-256 do diretório de regras)
- ReferenceImageCache + CompliancePromptBuilder (Prompt Caching)
- CloudFormation: ECS Task Def, Auto Scaling 1-10, SQS+DLQ
- Dockerfile.worker para ECS Fargate
- 773 testes passando (property, unit, integration)
</commit_message>
<xml_diff>
--- a/watchdog_rules/Comercializadores DGO y Amazon Prime - Websites.xlsx
+++ b/watchdog_rules/Comercializadores DGO y Amazon Prime - Websites.xlsx
@@ -1,20 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\DGO_SKY_WATCHDOG\watchdog_rules\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79661C94-B074-4FCE-93BB-DA1C1AB1988B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2684" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2741" uniqueCount="795">
   <si>
     <t>PAIS</t>
   </si>
@@ -136,7 +148,7 @@
     <t>LICOSINU S.A.S</t>
   </si>
   <si>
-    <t xml:space="preserve">LICOVACANA DEL PACIFICO S.A.S </t>
+    <t>LICOVACANA DEL PACIFICO S.A.S </t>
   </si>
   <si>
     <t>MPS MAYORISTA DE COLOMBIA SA</t>
@@ -304,7 +316,7 @@
     <t>CALOCASTRO &amp; PUBLICIDAD S.A.</t>
   </si>
   <si>
-    <t xml:space="preserve">GERARDO ORTIZ E HIJOS CIA LTDA </t>
+    <t>GERARDO ORTIZ E HIJOS CIA LTDA </t>
   </si>
   <si>
     <t>ZUKALO S.A. (SIIGO)</t>
@@ -2282,13 +2294,130 @@
   </si>
   <si>
     <t>https://dprimero.com/?srsltid=AfmBOoqszzPl68WCkYGkHa6JkR_Ot-X9rFebXVYdS5x3VTlxSVEQJY9M</t>
+  </si>
+  <si>
+    <t>Integrador</t>
+  </si>
+  <si>
+    <t>Parceiro</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>POWERNET SOLUTIONS</t>
+  </si>
+  <si>
+    <t>https://powernetsolutions.com.br/</t>
+  </si>
+  <si>
+    <t>AMIGO INTERNET</t>
+  </si>
+  <si>
+    <t>https://www.sejaamigo.com.br/tv-streaming</t>
+  </si>
+  <si>
+    <t>SEMPRE INTERNET</t>
+  </si>
+  <si>
+    <t>https://sempreinternet.com.br/</t>
+  </si>
+  <si>
+    <t>WECLIX</t>
+  </si>
+  <si>
+    <t>https://www.weclix.com.br/</t>
+  </si>
+  <si>
+    <t>DTEL TELECOM</t>
+  </si>
+  <si>
+    <t>https://dtel.com.br/home</t>
+  </si>
+  <si>
+    <t>CLICK.COM</t>
+  </si>
+  <si>
+    <t>https://provedorclick.com.br/</t>
+  </si>
+  <si>
+    <t>GRUPO JR TELECOM</t>
+  </si>
+  <si>
+    <t>https://netjrtelecom.com.br/</t>
+  </si>
+  <si>
+    <t>MUNDIAL TELECOM</t>
+  </si>
+  <si>
+    <t>https://mundialtelecom.net.br/</t>
+  </si>
+  <si>
+    <t>MAXX CONECTADO</t>
+  </si>
+  <si>
+    <t>https://maxxconectado.com.br/</t>
+  </si>
+  <si>
+    <t>DIGITAL NET MS</t>
+  </si>
+  <si>
+    <t>https://digitalnetms.com.br/</t>
+  </si>
+  <si>
+    <t>WORLDNET FIBRA</t>
+  </si>
+  <si>
+    <t>https://www.worldnetfibra.com.br/</t>
+  </si>
+  <si>
+    <t>SPEED TRAVEL</t>
+  </si>
+  <si>
+    <t>https://speedtravel.com.br/</t>
+  </si>
+  <si>
+    <t>ONNET</t>
+  </si>
+  <si>
+    <t>https://www.onnetmais.com.br/</t>
+  </si>
+  <si>
+    <t>FUTEL</t>
+  </si>
+  <si>
+    <t>https://futel.com.br/</t>
+  </si>
+  <si>
+    <t>DATANET</t>
+  </si>
+  <si>
+    <t>https://datanetprovedor.com.br/</t>
+  </si>
+  <si>
+    <t>ATEL</t>
+  </si>
+  <si>
+    <t>https://ateltelecom.com.br/</t>
+  </si>
+  <si>
+    <t>WORKSAT SERVIÇOS</t>
+  </si>
+  <si>
+    <t>https://worksattelecom.net.br/</t>
+  </si>
+  <si>
+    <t>UNISERVIÇOS</t>
+  </si>
+  <si>
+    <t>https://souuni.com/cidade/alvorada</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2351,12 +2480,21 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2364,13 +2502,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2408,7 +2554,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -2442,6 +2588,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2476,9 +2623,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2651,11 +2799,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H383"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2681,7 +2829,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2704,7 +2852,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2727,7 +2875,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2750,7 +2898,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2773,7 +2921,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2796,7 +2944,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2819,7 +2967,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2842,7 +2990,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2865,7 +3013,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2888,7 +3036,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -2911,7 +3059,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -2934,7 +3082,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -2957,7 +3105,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -2980,7 +3128,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -3003,7 +3151,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -3026,7 +3174,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -3049,7 +3197,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -3072,7 +3220,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -3095,7 +3243,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -3118,7 +3266,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -3141,7 +3289,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -3164,7 +3312,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -3187,7 +3335,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -3210,7 +3358,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -3233,7 +3381,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -3256,7 +3404,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -3279,7 +3427,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -3302,7 +3450,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -3325,7 +3473,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -3348,7 +3496,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -3371,7 +3519,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -3394,7 +3542,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -3417,7 +3565,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -3440,7 +3588,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -3463,7 +3611,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -3486,7 +3634,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -3509,7 +3657,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -3532,7 +3680,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -3555,7 +3703,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>8</v>
       </c>
@@ -3578,7 +3726,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -3601,7 +3749,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -3624,7 +3772,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>8</v>
       </c>
@@ -3647,7 +3795,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>8</v>
       </c>
@@ -3670,7 +3818,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -3693,7 +3841,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>8</v>
       </c>
@@ -3716,7 +3864,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -3739,7 +3887,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -3762,7 +3910,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -3785,7 +3933,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>8</v>
       </c>
@@ -3808,7 +3956,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>8</v>
       </c>
@@ -3831,7 +3979,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>8</v>
       </c>
@@ -3854,7 +4002,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -3877,7 +4025,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -3900,7 +4048,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>8</v>
       </c>
@@ -3923,7 +4071,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -3946,7 +4094,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>8</v>
       </c>
@@ -3969,7 +4117,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>8</v>
       </c>
@@ -3992,7 +4140,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -4015,7 +4163,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>8</v>
       </c>
@@ -4038,7 +4186,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>9</v>
       </c>
@@ -4061,7 +4209,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>9</v>
       </c>
@@ -4084,7 +4232,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>9</v>
       </c>
@@ -4107,7 +4255,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -4130,7 +4278,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>9</v>
       </c>
@@ -4153,7 +4301,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>9</v>
       </c>
@@ -4176,7 +4324,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>9</v>
       </c>
@@ -4199,7 +4347,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>9</v>
       </c>
@@ -4222,7 +4370,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>9</v>
       </c>
@@ -4245,7 +4393,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>9</v>
       </c>
@@ -4268,7 +4416,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>9</v>
       </c>
@@ -4291,7 +4439,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>9</v>
       </c>
@@ -4314,7 +4462,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>9</v>
       </c>
@@ -4337,7 +4485,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>9</v>
       </c>
@@ -4360,7 +4508,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>9</v>
       </c>
@@ -4383,7 +4531,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>9</v>
       </c>
@@ -4406,7 +4554,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>9</v>
       </c>
@@ -4429,7 +4577,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -4452,7 +4600,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>9</v>
       </c>
@@ -4475,7 +4623,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>9</v>
       </c>
@@ -4498,7 +4646,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>9</v>
       </c>
@@ -4521,7 +4669,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>9</v>
       </c>
@@ -4544,7 +4692,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>9</v>
       </c>
@@ -4567,7 +4715,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>9</v>
       </c>
@@ -4590,7 +4738,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>9</v>
       </c>
@@ -4613,7 +4761,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="86" spans="1:8">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>9</v>
       </c>
@@ -4636,7 +4784,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>10</v>
       </c>
@@ -4659,7 +4807,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>10</v>
       </c>
@@ -4682,7 +4830,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>10</v>
       </c>
@@ -4705,7 +4853,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>10</v>
       </c>
@@ -4728,7 +4876,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>10</v>
       </c>
@@ -4751,7 +4899,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>10</v>
       </c>
@@ -4774,7 +4922,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>10</v>
       </c>
@@ -4797,7 +4945,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>10</v>
       </c>
@@ -4820,7 +4968,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>10</v>
       </c>
@@ -4843,7 +4991,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="96" spans="1:8">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>10</v>
       </c>
@@ -4866,7 +5014,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="97" spans="1:8">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>10</v>
       </c>
@@ -4889,7 +5037,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="98" spans="1:8">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>10</v>
       </c>
@@ -4912,7 +5060,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="99" spans="1:8">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>10</v>
       </c>
@@ -4935,7 +5083,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="100" spans="1:8">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>10</v>
       </c>
@@ -4958,7 +5106,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="101" spans="1:8">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>10</v>
       </c>
@@ -4981,7 +5129,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="102" spans="1:8">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>10</v>
       </c>
@@ -5004,7 +5152,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="103" spans="1:8">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>11</v>
       </c>
@@ -5027,7 +5175,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="104" spans="1:8">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>12</v>
       </c>
@@ -5050,7 +5198,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="105" spans="1:8">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>12</v>
       </c>
@@ -5073,7 +5221,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="106" spans="1:8">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>13</v>
       </c>
@@ -5096,7 +5244,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="107" spans="1:8">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>13</v>
       </c>
@@ -5119,7 +5267,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="108" spans="1:8">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>13</v>
       </c>
@@ -5142,7 +5290,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="109" spans="1:8">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>13</v>
       </c>
@@ -5165,7 +5313,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="110" spans="1:8">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>13</v>
       </c>
@@ -5188,7 +5336,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="111" spans="1:8">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>13</v>
       </c>
@@ -5211,7 +5359,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="112" spans="1:8">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>13</v>
       </c>
@@ -5234,7 +5382,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="113" spans="1:8">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>13</v>
       </c>
@@ -5257,7 +5405,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="114" spans="1:8">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>8</v>
       </c>
@@ -5280,7 +5428,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="115" spans="1:8">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>8</v>
       </c>
@@ -5306,7 +5454,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>8</v>
       </c>
@@ -5329,7 +5477,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="117" spans="1:8">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>8</v>
       </c>
@@ -5352,7 +5500,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="118" spans="1:8">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>8</v>
       </c>
@@ -5375,7 +5523,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="119" spans="1:8">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>8</v>
       </c>
@@ -5398,7 +5546,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="120" spans="1:8">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>8</v>
       </c>
@@ -5421,7 +5569,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="121" spans="1:8">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>8</v>
       </c>
@@ -5444,7 +5592,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="122" spans="1:8">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>8</v>
       </c>
@@ -5467,7 +5615,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="123" spans="1:8">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>8</v>
       </c>
@@ -5490,7 +5638,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="124" spans="1:8">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>8</v>
       </c>
@@ -5513,7 +5661,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="125" spans="1:8">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>8</v>
       </c>
@@ -5536,7 +5684,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="126" spans="1:8">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>8</v>
       </c>
@@ -5559,7 +5707,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="127" spans="1:8">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>8</v>
       </c>
@@ -5582,7 +5730,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="128" spans="1:8">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>8</v>
       </c>
@@ -5605,7 +5753,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="129" spans="1:8">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>8</v>
       </c>
@@ -5628,7 +5776,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="130" spans="1:8">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>8</v>
       </c>
@@ -5651,7 +5799,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="131" spans="1:8">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>8</v>
       </c>
@@ -5674,7 +5822,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="132" spans="1:8">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>8</v>
       </c>
@@ -5697,7 +5845,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="133" spans="1:8">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>8</v>
       </c>
@@ -5720,7 +5868,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="134" spans="1:8">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>8</v>
       </c>
@@ -5743,7 +5891,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="135" spans="1:8">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>8</v>
       </c>
@@ -5766,7 +5914,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="136" spans="1:8">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>8</v>
       </c>
@@ -5789,7 +5937,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="137" spans="1:8">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>8</v>
       </c>
@@ -5812,7 +5960,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="138" spans="1:8">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>8</v>
       </c>
@@ -5835,7 +5983,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="139" spans="1:8">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>8</v>
       </c>
@@ -5858,7 +6006,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="140" spans="1:8">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>8</v>
       </c>
@@ -5881,7 +6029,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="141" spans="1:8">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>8</v>
       </c>
@@ -5904,7 +6052,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="142" spans="1:8">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>8</v>
       </c>
@@ -5927,7 +6075,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="143" spans="1:8">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>8</v>
       </c>
@@ -5950,7 +6098,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="144" spans="1:8">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>8</v>
       </c>
@@ -5973,7 +6121,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="145" spans="1:8">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>8</v>
       </c>
@@ -5996,7 +6144,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="146" spans="1:8">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>8</v>
       </c>
@@ -6019,7 +6167,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="147" spans="1:8">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>8</v>
       </c>
@@ -6042,7 +6190,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="148" spans="1:8">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>8</v>
       </c>
@@ -6065,7 +6213,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="149" spans="1:8">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>8</v>
       </c>
@@ -6088,7 +6236,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="150" spans="1:8">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>8</v>
       </c>
@@ -6111,7 +6259,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="151" spans="1:8">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>8</v>
       </c>
@@ -6134,7 +6282,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="152" spans="1:8">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>8</v>
       </c>
@@ -6157,7 +6305,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="153" spans="1:8">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>8</v>
       </c>
@@ -6180,7 +6328,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="154" spans="1:8">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>8</v>
       </c>
@@ -6203,7 +6351,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="155" spans="1:8">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>8</v>
       </c>
@@ -6226,7 +6374,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="156" spans="1:8">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>8</v>
       </c>
@@ -6249,7 +6397,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="157" spans="1:8">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>8</v>
       </c>
@@ -6272,7 +6420,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="158" spans="1:8">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>8</v>
       </c>
@@ -6295,7 +6443,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="159" spans="1:8">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>8</v>
       </c>
@@ -6318,7 +6466,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="160" spans="1:8">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>8</v>
       </c>
@@ -6341,7 +6489,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="161" spans="1:8">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>8</v>
       </c>
@@ -6364,7 +6512,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="162" spans="1:8">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>8</v>
       </c>
@@ -6387,7 +6535,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="163" spans="1:8">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>8</v>
       </c>
@@ -6410,7 +6558,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="164" spans="1:8">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>8</v>
       </c>
@@ -6433,7 +6581,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="165" spans="1:8">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>8</v>
       </c>
@@ -6456,7 +6604,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="166" spans="1:8">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>8</v>
       </c>
@@ -6479,7 +6627,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="167" spans="1:8">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>8</v>
       </c>
@@ -6502,7 +6650,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="168" spans="1:8">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>8</v>
       </c>
@@ -6525,7 +6673,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="169" spans="1:8">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>8</v>
       </c>
@@ -6548,7 +6696,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="170" spans="1:8">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>8</v>
       </c>
@@ -6571,7 +6719,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="171" spans="1:8">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>8</v>
       </c>
@@ -6594,7 +6742,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="172" spans="1:8">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>8</v>
       </c>
@@ -6617,7 +6765,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="173" spans="1:8">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>8</v>
       </c>
@@ -6640,7 +6788,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="174" spans="1:8">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>8</v>
       </c>
@@ -6663,7 +6811,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="175" spans="1:8">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>8</v>
       </c>
@@ -6686,7 +6834,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="176" spans="1:8">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>10</v>
       </c>
@@ -6709,7 +6857,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="177" spans="1:8">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>10</v>
       </c>
@@ -6732,7 +6880,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="178" spans="1:8">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>10</v>
       </c>
@@ -6758,7 +6906,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="179" spans="1:8">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>10</v>
       </c>
@@ -6781,7 +6929,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="180" spans="1:8">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>10</v>
       </c>
@@ -6804,7 +6952,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="181" spans="1:8">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>10</v>
       </c>
@@ -6827,7 +6975,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="182" spans="1:8">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>10</v>
       </c>
@@ -6850,7 +6998,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="183" spans="1:8">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>10</v>
       </c>
@@ -6873,7 +7021,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="184" spans="1:8">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>10</v>
       </c>
@@ -6896,7 +7044,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="185" spans="1:8">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>10</v>
       </c>
@@ -6919,7 +7067,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="186" spans="1:8">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>10</v>
       </c>
@@ -6942,7 +7090,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="187" spans="1:8">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>10</v>
       </c>
@@ -6965,7 +7113,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="188" spans="1:8">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>8</v>
       </c>
@@ -6988,7 +7136,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="189" spans="1:8">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>8</v>
       </c>
@@ -7011,7 +7159,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="190" spans="1:8">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>8</v>
       </c>
@@ -7034,7 +7182,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="191" spans="1:8">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>8</v>
       </c>
@@ -7057,7 +7205,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="192" spans="1:8">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>8</v>
       </c>
@@ -7080,7 +7228,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="193" spans="1:8">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>8</v>
       </c>
@@ -7103,7 +7251,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="194" spans="1:8">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>8</v>
       </c>
@@ -7126,7 +7274,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="195" spans="1:8">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>9</v>
       </c>
@@ -7149,7 +7297,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="196" spans="1:8">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>10</v>
       </c>
@@ -7172,7 +7320,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="197" spans="1:8">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>8</v>
       </c>
@@ -7195,7 +7343,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="198" spans="1:8">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>10</v>
       </c>
@@ -7218,7 +7366,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="199" spans="1:8">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>8</v>
       </c>
@@ -7241,7 +7389,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="200" spans="1:8">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>9</v>
       </c>
@@ -7264,7 +7412,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="201" spans="1:8">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>8</v>
       </c>
@@ -7287,7 +7435,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="202" spans="1:8">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>8</v>
       </c>
@@ -7310,7 +7458,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="203" spans="1:8">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>8</v>
       </c>
@@ -7333,7 +7481,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="204" spans="1:8">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>8</v>
       </c>
@@ -7356,7 +7504,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="205" spans="1:8">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>9</v>
       </c>
@@ -7379,7 +7527,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="206" spans="1:8">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>8</v>
       </c>
@@ -7402,7 +7550,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="207" spans="1:8">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>9</v>
       </c>
@@ -7425,7 +7573,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="208" spans="1:8">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>8</v>
       </c>
@@ -7448,7 +7596,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="209" spans="1:8">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>8</v>
       </c>
@@ -7471,7 +7619,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="210" spans="1:8">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>9</v>
       </c>
@@ -7494,7 +7642,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="211" spans="1:8">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>8</v>
       </c>
@@ -7517,7 +7665,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="212" spans="1:8">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>8</v>
       </c>
@@ -7540,7 +7688,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="213" spans="1:8">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>9</v>
       </c>
@@ -7563,7 +7711,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="214" spans="1:8">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>8</v>
       </c>
@@ -7586,7 +7734,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="215" spans="1:8">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>9</v>
       </c>
@@ -7609,7 +7757,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="216" spans="1:8">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>8</v>
       </c>
@@ -7632,7 +7780,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="217" spans="1:8">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>8</v>
       </c>
@@ -7655,7 +7803,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="218" spans="1:8">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>8</v>
       </c>
@@ -7678,7 +7826,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="219" spans="1:8">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>8</v>
       </c>
@@ -7701,7 +7849,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="220" spans="1:8">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>9</v>
       </c>
@@ -7724,7 +7872,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="221" spans="1:8">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>8</v>
       </c>
@@ -7747,7 +7895,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="222" spans="1:8">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>8</v>
       </c>
@@ -7770,7 +7918,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="223" spans="1:8">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>8</v>
       </c>
@@ -7793,7 +7941,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="224" spans="1:8">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>8</v>
       </c>
@@ -7816,7 +7964,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="225" spans="1:8">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>8</v>
       </c>
@@ -7839,7 +7987,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="226" spans="1:8">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>8</v>
       </c>
@@ -7862,7 +8010,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="227" spans="1:8">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>9</v>
       </c>
@@ -7885,7 +8033,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="228" spans="1:8">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>10</v>
       </c>
@@ -7908,7 +8056,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="229" spans="1:8">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>8</v>
       </c>
@@ -7931,7 +8079,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="230" spans="1:8">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>8</v>
       </c>
@@ -7954,7 +8102,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="231" spans="1:8">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>8</v>
       </c>
@@ -7977,7 +8125,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="232" spans="1:8">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>8</v>
       </c>
@@ -8000,7 +8148,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="233" spans="1:8">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>8</v>
       </c>
@@ -8023,7 +8171,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="234" spans="1:8">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>8</v>
       </c>
@@ -8046,7 +8194,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="235" spans="1:8">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>9</v>
       </c>
@@ -8069,7 +8217,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="236" spans="1:8">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>9</v>
       </c>
@@ -8092,7 +8240,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="237" spans="1:8">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>8</v>
       </c>
@@ -8115,7 +8263,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="238" spans="1:8">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>8</v>
       </c>
@@ -8138,7 +8286,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="239" spans="1:8">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>8</v>
       </c>
@@ -8161,7 +8309,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="240" spans="1:8">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>8</v>
       </c>
@@ -8184,7 +8332,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="241" spans="1:8">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>8</v>
       </c>
@@ -8207,7 +8355,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="242" spans="1:8">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>8</v>
       </c>
@@ -8230,7 +8378,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="243" spans="1:8">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>9</v>
       </c>
@@ -8253,7 +8401,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="244" spans="1:8">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>9</v>
       </c>
@@ -8276,7 +8424,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="245" spans="1:8">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>10</v>
       </c>
@@ -8299,7 +8447,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="246" spans="1:8">
+    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>10</v>
       </c>
@@ -8322,7 +8470,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="247" spans="1:8">
+    <row r="247" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>8</v>
       </c>
@@ -8345,7 +8493,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="248" spans="1:8">
+    <row r="248" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>8</v>
       </c>
@@ -8368,7 +8516,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="249" spans="1:8">
+    <row r="249" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>8</v>
       </c>
@@ -8391,7 +8539,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="250" spans="1:8">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>8</v>
       </c>
@@ -8414,7 +8562,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="251" spans="1:8">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>8</v>
       </c>
@@ -8437,7 +8585,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="252" spans="1:8">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>8</v>
       </c>
@@ -8460,7 +8608,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="253" spans="1:8">
+    <row r="253" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>8</v>
       </c>
@@ -8483,7 +8631,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="254" spans="1:8">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>8</v>
       </c>
@@ -8506,7 +8654,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="255" spans="1:8">
+    <row r="255" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>8</v>
       </c>
@@ -8529,7 +8677,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="256" spans="1:8">
+    <row r="256" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>8</v>
       </c>
@@ -8552,7 +8700,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="257" spans="1:8">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>9</v>
       </c>
@@ -8575,7 +8723,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="258" spans="1:8">
+    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>8</v>
       </c>
@@ -8598,7 +8746,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="259" spans="1:8">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>8</v>
       </c>
@@ -8621,7 +8769,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="260" spans="1:8">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>8</v>
       </c>
@@ -8644,7 +8792,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="261" spans="1:8">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>9</v>
       </c>
@@ -8667,7 +8815,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="262" spans="1:8">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>8</v>
       </c>
@@ -8690,7 +8838,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="263" spans="1:8">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>8</v>
       </c>
@@ -8713,7 +8861,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="264" spans="1:8">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>9</v>
       </c>
@@ -8736,7 +8884,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="265" spans="1:8">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>9</v>
       </c>
@@ -8759,7 +8907,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="266" spans="1:8">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>8</v>
       </c>
@@ -8782,7 +8930,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="267" spans="1:8">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>8</v>
       </c>
@@ -8805,7 +8953,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="268" spans="1:8">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>8</v>
       </c>
@@ -8828,7 +8976,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="269" spans="1:8">
+    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>8</v>
       </c>
@@ -8851,7 +8999,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="270" spans="1:8">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>8</v>
       </c>
@@ -8874,7 +9022,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="271" spans="1:8">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>8</v>
       </c>
@@ -8897,7 +9045,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="272" spans="1:8">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>8</v>
       </c>
@@ -8920,7 +9068,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="273" spans="1:8">
+    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>8</v>
       </c>
@@ -8943,7 +9091,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="274" spans="1:8">
+    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>8</v>
       </c>
@@ -8966,7 +9114,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="275" spans="1:8">
+    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>8</v>
       </c>
@@ -8989,7 +9137,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="276" spans="1:8">
+    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>9</v>
       </c>
@@ -9012,7 +9160,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="277" spans="1:8">
+    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>8</v>
       </c>
@@ -9035,7 +9183,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="278" spans="1:8">
+    <row r="278" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>9</v>
       </c>
@@ -9058,7 +9206,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="279" spans="1:8">
+    <row r="279" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>8</v>
       </c>
@@ -9081,7 +9229,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="280" spans="1:8">
+    <row r="280" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>9</v>
       </c>
@@ -9104,7 +9252,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="281" spans="1:8">
+    <row r="281" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>11</v>
       </c>
@@ -9127,7 +9275,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="282" spans="1:8">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>11</v>
       </c>
@@ -9150,7 +9298,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="283" spans="1:8">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>11</v>
       </c>
@@ -9173,7 +9321,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="284" spans="1:8">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>11</v>
       </c>
@@ -9196,7 +9344,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="285" spans="1:8">
+    <row r="285" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>11</v>
       </c>
@@ -9219,7 +9367,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="286" spans="1:8">
+    <row r="286" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>11</v>
       </c>
@@ -9242,7 +9390,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="287" spans="1:8">
+    <row r="287" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>11</v>
       </c>
@@ -9265,7 +9413,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="288" spans="1:8">
+    <row r="288" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>11</v>
       </c>
@@ -9288,7 +9436,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="289" spans="1:8">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>11</v>
       </c>
@@ -9311,7 +9459,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="290" spans="1:8">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>11</v>
       </c>
@@ -9334,7 +9482,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="291" spans="1:8">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>11</v>
       </c>
@@ -9357,7 +9505,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="292" spans="1:8">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>11</v>
       </c>
@@ -9380,7 +9528,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="293" spans="1:8">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>11</v>
       </c>
@@ -9403,7 +9551,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="294" spans="1:8">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>11</v>
       </c>
@@ -9426,7 +9574,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="295" spans="1:8">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>11</v>
       </c>
@@ -9449,7 +9597,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="296" spans="1:8">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>11</v>
       </c>
@@ -9472,7 +9620,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="297" spans="1:8">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>11</v>
       </c>
@@ -9495,7 +9643,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="298" spans="1:8">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>11</v>
       </c>
@@ -9518,7 +9666,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="299" spans="1:8">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>11</v>
       </c>
@@ -9541,7 +9689,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="300" spans="1:8">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>11</v>
       </c>
@@ -9564,7 +9712,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="301" spans="1:8">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>11</v>
       </c>
@@ -9587,7 +9735,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="302" spans="1:8">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>11</v>
       </c>
@@ -9610,7 +9758,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="303" spans="1:8">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>11</v>
       </c>
@@ -9633,7 +9781,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="304" spans="1:8">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>11</v>
       </c>
@@ -9656,7 +9804,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="305" spans="1:8">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>11</v>
       </c>
@@ -9679,7 +9827,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="306" spans="1:8">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>11</v>
       </c>
@@ -9702,7 +9850,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="307" spans="1:8">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>11</v>
       </c>
@@ -9725,7 +9873,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="308" spans="1:8">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>11</v>
       </c>
@@ -9748,7 +9896,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="309" spans="1:8">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>11</v>
       </c>
@@ -9771,7 +9919,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="310" spans="1:8">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>11</v>
       </c>
@@ -9794,7 +9942,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="311" spans="1:8">
+    <row r="311" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>11</v>
       </c>
@@ -9817,7 +9965,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="312" spans="1:8">
+    <row r="312" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>11</v>
       </c>
@@ -9840,7 +9988,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="313" spans="1:8">
+    <row r="313" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>11</v>
       </c>
@@ -9863,7 +10011,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="314" spans="1:8">
+    <row r="314" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>11</v>
       </c>
@@ -9886,7 +10034,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="315" spans="1:8">
+    <row r="315" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>11</v>
       </c>
@@ -9909,7 +10057,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="316" spans="1:8">
+    <row r="316" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>11</v>
       </c>
@@ -9932,7 +10080,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="317" spans="1:8">
+    <row r="317" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>11</v>
       </c>
@@ -9955,7 +10103,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="318" spans="1:8">
+    <row r="318" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>11</v>
       </c>
@@ -9978,7 +10126,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="319" spans="1:8">
+    <row r="319" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>11</v>
       </c>
@@ -10001,7 +10149,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="320" spans="1:8">
+    <row r="320" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>11</v>
       </c>
@@ -10024,7 +10172,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="321" spans="1:8">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>11</v>
       </c>
@@ -10047,7 +10195,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="322" spans="1:8">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>11</v>
       </c>
@@ -10070,7 +10218,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="323" spans="1:8">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>11</v>
       </c>
@@ -10093,7 +10241,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="324" spans="1:8">
+    <row r="324" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>11</v>
       </c>
@@ -10116,7 +10264,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="325" spans="1:8">
+    <row r="325" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>11</v>
       </c>
@@ -10139,7 +10287,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="326" spans="1:8">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>11</v>
       </c>
@@ -10162,7 +10310,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="327" spans="1:8">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>11</v>
       </c>
@@ -10185,7 +10333,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="328" spans="1:8">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>11</v>
       </c>
@@ -10208,7 +10356,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="329" spans="1:8">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>11</v>
       </c>
@@ -10231,7 +10379,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="330" spans="1:8">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>11</v>
       </c>
@@ -10254,7 +10402,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="331" spans="1:8">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>11</v>
       </c>
@@ -10277,7 +10425,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="332" spans="1:8">
+    <row r="332" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>11</v>
       </c>
@@ -10300,7 +10448,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="333" spans="1:8">
+    <row r="333" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>11</v>
       </c>
@@ -10323,7 +10471,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="334" spans="1:8">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>11</v>
       </c>
@@ -10346,7 +10494,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="335" spans="1:8">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>11</v>
       </c>
@@ -10369,7 +10517,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="336" spans="1:8">
+    <row r="336" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>11</v>
       </c>
@@ -10392,7 +10540,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="337" spans="1:8">
+    <row r="337" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>11</v>
       </c>
@@ -10415,7 +10563,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="338" spans="1:8">
+    <row r="338" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>11</v>
       </c>
@@ -10438,7 +10586,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="339" spans="1:8">
+    <row r="339" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>11</v>
       </c>
@@ -10461,7 +10609,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="340" spans="1:8">
+    <row r="340" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>11</v>
       </c>
@@ -10484,7 +10632,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="341" spans="1:8">
+    <row r="341" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>11</v>
       </c>
@@ -10507,7 +10655,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="342" spans="1:8">
+    <row r="342" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>11</v>
       </c>
@@ -10530,7 +10678,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="343" spans="1:8">
+    <row r="343" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>11</v>
       </c>
@@ -10553,7 +10701,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="344" spans="1:8">
+    <row r="344" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>11</v>
       </c>
@@ -10576,7 +10724,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="345" spans="1:8">
+    <row r="345" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>12</v>
       </c>
@@ -10599,7 +10747,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="346" spans="1:8">
+    <row r="346" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>12</v>
       </c>
@@ -10622,7 +10770,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="347" spans="1:8">
+    <row r="347" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>12</v>
       </c>
@@ -10645,7 +10793,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="348" spans="1:8">
+    <row r="348" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>8</v>
       </c>
@@ -10668,7 +10816,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="349" spans="1:8">
+    <row r="349" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>8</v>
       </c>
@@ -10691,7 +10839,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="350" spans="1:8">
+    <row r="350" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>8</v>
       </c>
@@ -10714,7 +10862,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="351" spans="1:8">
+    <row r="351" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>8</v>
       </c>
@@ -10737,7 +10885,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="352" spans="1:8">
+    <row r="352" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>8</v>
       </c>
@@ -10760,7 +10908,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="353" spans="1:8">
+    <row r="353" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>8</v>
       </c>
@@ -10783,7 +10931,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="354" spans="1:8">
+    <row r="354" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>8</v>
       </c>
@@ -10806,7 +10954,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="355" spans="1:8">
+    <row r="355" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>8</v>
       </c>
@@ -10829,7 +10977,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="356" spans="1:8">
+    <row r="356" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>8</v>
       </c>
@@ -10852,7 +11000,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="357" spans="1:8">
+    <row r="357" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>8</v>
       </c>
@@ -10875,7 +11023,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="358" spans="1:8">
+    <row r="358" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>8</v>
       </c>
@@ -10898,7 +11046,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="359" spans="1:8">
+    <row r="359" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>8</v>
       </c>
@@ -10921,7 +11069,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="360" spans="1:8">
+    <row r="360" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>8</v>
       </c>
@@ -10944,7 +11092,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="361" spans="1:8">
+    <row r="361" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>8</v>
       </c>
@@ -10967,7 +11115,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="362" spans="1:8">
+    <row r="362" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>8</v>
       </c>
@@ -10990,7 +11138,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="363" spans="1:8">
+    <row r="363" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>8</v>
       </c>
@@ -11013,7 +11161,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="364" spans="1:8">
+    <row r="364" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>8</v>
       </c>
@@ -11036,7 +11184,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="365" spans="1:8">
+    <row r="365" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
         <v>8</v>
       </c>
@@ -11059,7 +11207,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="366" spans="1:8">
+    <row r="366" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
         <v>8</v>
       </c>
@@ -11082,7 +11230,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="367" spans="1:8">
+    <row r="367" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
         <v>8</v>
       </c>
@@ -11105,7 +11253,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="368" spans="1:8">
+    <row r="368" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
         <v>8</v>
       </c>
@@ -11128,7 +11276,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="369" spans="1:8">
+    <row r="369" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
         <v>8</v>
       </c>
@@ -11151,7 +11299,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="370" spans="1:8">
+    <row r="370" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
         <v>8</v>
       </c>
@@ -11174,7 +11322,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="371" spans="1:8">
+    <row r="371" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
         <v>8</v>
       </c>
@@ -11197,7 +11345,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="372" spans="1:8">
+    <row r="372" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
         <v>8</v>
       </c>
@@ -11220,7 +11368,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="373" spans="1:8">
+    <row r="373" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
         <v>8</v>
       </c>
@@ -11243,7 +11391,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="374" spans="1:8">
+    <row r="374" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
         <v>8</v>
       </c>
@@ -11266,7 +11414,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="375" spans="1:8">
+    <row r="375" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
         <v>8</v>
       </c>
@@ -11289,7 +11437,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="376" spans="1:8">
+    <row r="376" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
         <v>8</v>
       </c>
@@ -11312,7 +11460,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="377" spans="1:8">
+    <row r="377" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
         <v>8</v>
       </c>
@@ -11335,7 +11483,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="378" spans="1:8">
+    <row r="378" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
         <v>8</v>
       </c>
@@ -11358,7 +11506,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="379" spans="1:8">
+    <row r="379" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
         <v>8</v>
       </c>
@@ -11381,7 +11529,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="380" spans="1:8">
+    <row r="380" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
         <v>8</v>
       </c>
@@ -11404,7 +11552,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="381" spans="1:8">
+    <row r="381" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
         <v>8</v>
       </c>
@@ -11427,7 +11575,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="382" spans="1:8">
+    <row r="382" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
         <v>8</v>
       </c>
@@ -11450,7 +11598,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="383" spans="1:8">
+    <row r="383" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
         <v>8</v>
       </c>
@@ -11475,388 +11623,630 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1"/>
-    <hyperlink ref="H3" r:id="rId2"/>
-    <hyperlink ref="H4" r:id="rId3"/>
-    <hyperlink ref="H5" r:id="rId4"/>
-    <hyperlink ref="H6" r:id="rId5"/>
-    <hyperlink ref="H7" r:id="rId6"/>
-    <hyperlink ref="H8" r:id="rId7"/>
-    <hyperlink ref="H9" r:id="rId8"/>
-    <hyperlink ref="H10" r:id="rId9"/>
-    <hyperlink ref="H11" r:id="rId10"/>
-    <hyperlink ref="H12" r:id="rId11"/>
-    <hyperlink ref="H13" r:id="rId12"/>
-    <hyperlink ref="H14" r:id="rId13"/>
-    <hyperlink ref="H15" r:id="rId14"/>
-    <hyperlink ref="H16" r:id="rId15"/>
-    <hyperlink ref="H17" r:id="rId16"/>
-    <hyperlink ref="H18" r:id="rId17"/>
-    <hyperlink ref="H19" r:id="rId18"/>
-    <hyperlink ref="H20" r:id="rId19"/>
-    <hyperlink ref="H21" r:id="rId20"/>
-    <hyperlink ref="H22" r:id="rId21"/>
-    <hyperlink ref="H23" r:id="rId22"/>
-    <hyperlink ref="H24" r:id="rId23"/>
-    <hyperlink ref="H25" r:id="rId24"/>
-    <hyperlink ref="H26" r:id="rId25"/>
-    <hyperlink ref="H27" r:id="rId26"/>
-    <hyperlink ref="H28" r:id="rId27"/>
-    <hyperlink ref="H29" r:id="rId28"/>
-    <hyperlink ref="H30" r:id="rId29"/>
-    <hyperlink ref="H31" r:id="rId30"/>
-    <hyperlink ref="H32" r:id="rId31"/>
-    <hyperlink ref="H33" r:id="rId32"/>
-    <hyperlink ref="H34" r:id="rId33"/>
-    <hyperlink ref="H35" r:id="rId34"/>
-    <hyperlink ref="H36" r:id="rId35"/>
-    <hyperlink ref="H37" r:id="rId36"/>
-    <hyperlink ref="H38" r:id="rId37"/>
-    <hyperlink ref="H39" r:id="rId38"/>
-    <hyperlink ref="H40" r:id="rId39"/>
-    <hyperlink ref="H41" r:id="rId40"/>
-    <hyperlink ref="H42" r:id="rId41"/>
-    <hyperlink ref="H43" r:id="rId42"/>
-    <hyperlink ref="H44" r:id="rId43"/>
-    <hyperlink ref="H45" r:id="rId44"/>
-    <hyperlink ref="H46" r:id="rId45"/>
-    <hyperlink ref="H47" r:id="rId46"/>
-    <hyperlink ref="H48" r:id="rId47"/>
-    <hyperlink ref="H49" r:id="rId48"/>
-    <hyperlink ref="H50" r:id="rId49"/>
-    <hyperlink ref="H51" r:id="rId50"/>
-    <hyperlink ref="H52" r:id="rId51"/>
-    <hyperlink ref="H53" r:id="rId52"/>
-    <hyperlink ref="H54" r:id="rId53"/>
-    <hyperlink ref="H55" r:id="rId54"/>
-    <hyperlink ref="H56" r:id="rId55"/>
-    <hyperlink ref="H57" r:id="rId56"/>
-    <hyperlink ref="H58" r:id="rId57"/>
-    <hyperlink ref="H59" r:id="rId58"/>
-    <hyperlink ref="H60" r:id="rId59"/>
-    <hyperlink ref="H61" r:id="rId60"/>
-    <hyperlink ref="H62" r:id="rId61"/>
-    <hyperlink ref="H63" r:id="rId62"/>
-    <hyperlink ref="H64" r:id="rId63"/>
-    <hyperlink ref="H65" r:id="rId64"/>
-    <hyperlink ref="H66" r:id="rId65"/>
-    <hyperlink ref="H67" r:id="rId66"/>
-    <hyperlink ref="H68" r:id="rId67"/>
-    <hyperlink ref="H69" r:id="rId68"/>
-    <hyperlink ref="H70" r:id="rId69"/>
-    <hyperlink ref="H71" r:id="rId70"/>
-    <hyperlink ref="H72" r:id="rId71"/>
-    <hyperlink ref="H73" r:id="rId72"/>
-    <hyperlink ref="H74" r:id="rId73"/>
-    <hyperlink ref="H75" r:id="rId74"/>
-    <hyperlink ref="H76" r:id="rId75"/>
-    <hyperlink ref="H77" r:id="rId76"/>
-    <hyperlink ref="H78" r:id="rId77"/>
-    <hyperlink ref="H79" r:id="rId78"/>
-    <hyperlink ref="H80" r:id="rId79"/>
-    <hyperlink ref="H81" r:id="rId80"/>
-    <hyperlink ref="H82" r:id="rId81"/>
-    <hyperlink ref="H83" r:id="rId82"/>
-    <hyperlink ref="H84" r:id="rId83"/>
-    <hyperlink ref="H85" r:id="rId84"/>
-    <hyperlink ref="H86" r:id="rId85"/>
-    <hyperlink ref="H87" r:id="rId86"/>
-    <hyperlink ref="H88" r:id="rId87"/>
-    <hyperlink ref="H89" r:id="rId88"/>
-    <hyperlink ref="H90" r:id="rId89"/>
-    <hyperlink ref="H91" r:id="rId90"/>
-    <hyperlink ref="H92" r:id="rId91"/>
-    <hyperlink ref="H93" r:id="rId92"/>
-    <hyperlink ref="H94" r:id="rId93"/>
-    <hyperlink ref="H95" r:id="rId94"/>
-    <hyperlink ref="H96" r:id="rId95"/>
-    <hyperlink ref="H97" r:id="rId96"/>
-    <hyperlink ref="H98" r:id="rId97"/>
-    <hyperlink ref="H99" r:id="rId98"/>
-    <hyperlink ref="H100" r:id="rId99"/>
-    <hyperlink ref="H101" r:id="rId100"/>
-    <hyperlink ref="H102" r:id="rId101"/>
-    <hyperlink ref="H103" r:id="rId102"/>
-    <hyperlink ref="H104" r:id="rId103"/>
-    <hyperlink ref="H105" r:id="rId104"/>
-    <hyperlink ref="H106" r:id="rId105"/>
-    <hyperlink ref="H107" r:id="rId106"/>
-    <hyperlink ref="H108" r:id="rId107"/>
-    <hyperlink ref="H109" r:id="rId108"/>
-    <hyperlink ref="H110" r:id="rId109"/>
-    <hyperlink ref="H111" r:id="rId110"/>
-    <hyperlink ref="H112" r:id="rId111"/>
-    <hyperlink ref="H113" r:id="rId112"/>
-    <hyperlink ref="H114" r:id="rId113"/>
-    <hyperlink ref="H115" r:id="rId114"/>
-    <hyperlink ref="H116" r:id="rId115"/>
-    <hyperlink ref="H117" r:id="rId116"/>
-    <hyperlink ref="H118" r:id="rId117"/>
-    <hyperlink ref="H119" r:id="rId118"/>
-    <hyperlink ref="H120" r:id="rId119"/>
-    <hyperlink ref="H121" r:id="rId120"/>
-    <hyperlink ref="H122" r:id="rId121"/>
-    <hyperlink ref="H123" r:id="rId122"/>
-    <hyperlink ref="H124" r:id="rId123"/>
-    <hyperlink ref="H125" r:id="rId124"/>
-    <hyperlink ref="H126" r:id="rId125"/>
-    <hyperlink ref="H127" r:id="rId126"/>
-    <hyperlink ref="H128" r:id="rId127"/>
-    <hyperlink ref="H129" r:id="rId128"/>
-    <hyperlink ref="H130" r:id="rId129"/>
-    <hyperlink ref="H131" r:id="rId130"/>
-    <hyperlink ref="H132" r:id="rId131"/>
-    <hyperlink ref="H133" r:id="rId132"/>
-    <hyperlink ref="H134" r:id="rId133"/>
-    <hyperlink ref="H135" r:id="rId134"/>
-    <hyperlink ref="H136" r:id="rId135"/>
-    <hyperlink ref="H137" r:id="rId136"/>
-    <hyperlink ref="H138" r:id="rId137"/>
-    <hyperlink ref="H139" r:id="rId138"/>
-    <hyperlink ref="H140" r:id="rId139"/>
-    <hyperlink ref="H141" r:id="rId140"/>
-    <hyperlink ref="H142" r:id="rId141"/>
-    <hyperlink ref="H143" r:id="rId142"/>
-    <hyperlink ref="H144" r:id="rId143"/>
-    <hyperlink ref="H145" r:id="rId144"/>
-    <hyperlink ref="H146" r:id="rId145"/>
-    <hyperlink ref="H147" r:id="rId146"/>
-    <hyperlink ref="H148" r:id="rId147"/>
-    <hyperlink ref="H149" r:id="rId148"/>
-    <hyperlink ref="H150" r:id="rId149"/>
-    <hyperlink ref="H151" r:id="rId150"/>
-    <hyperlink ref="H152" r:id="rId151"/>
-    <hyperlink ref="H153" r:id="rId152"/>
-    <hyperlink ref="H154" r:id="rId153"/>
-    <hyperlink ref="H155" r:id="rId154"/>
-    <hyperlink ref="H156" r:id="rId155"/>
-    <hyperlink ref="H157" r:id="rId156"/>
-    <hyperlink ref="H158" r:id="rId157"/>
-    <hyperlink ref="H159" r:id="rId158"/>
-    <hyperlink ref="H160" r:id="rId159"/>
-    <hyperlink ref="H161" r:id="rId160"/>
-    <hyperlink ref="H162" r:id="rId161"/>
-    <hyperlink ref="H163" r:id="rId162"/>
-    <hyperlink ref="H164" r:id="rId163"/>
-    <hyperlink ref="H165" r:id="rId164"/>
-    <hyperlink ref="H166" r:id="rId165"/>
-    <hyperlink ref="H167" r:id="rId166"/>
-    <hyperlink ref="H168" r:id="rId167"/>
-    <hyperlink ref="H169" r:id="rId168"/>
-    <hyperlink ref="H170" r:id="rId169"/>
-    <hyperlink ref="H171" r:id="rId170"/>
-    <hyperlink ref="H172" r:id="rId171"/>
-    <hyperlink ref="H173" r:id="rId172"/>
-    <hyperlink ref="H174" r:id="rId173"/>
-    <hyperlink ref="H175" r:id="rId174"/>
-    <hyperlink ref="H176" r:id="rId175"/>
-    <hyperlink ref="H177" r:id="rId176"/>
-    <hyperlink ref="H178" r:id="rId177"/>
-    <hyperlink ref="H179" r:id="rId178"/>
-    <hyperlink ref="H180" r:id="rId179"/>
-    <hyperlink ref="H181" r:id="rId180"/>
-    <hyperlink ref="H182" r:id="rId181"/>
-    <hyperlink ref="H183" r:id="rId182"/>
-    <hyperlink ref="H184" r:id="rId183"/>
-    <hyperlink ref="H185" r:id="rId184"/>
-    <hyperlink ref="H186" r:id="rId185"/>
-    <hyperlink ref="H187" r:id="rId186"/>
-    <hyperlink ref="H188" r:id="rId187"/>
-    <hyperlink ref="H189" r:id="rId188"/>
-    <hyperlink ref="H190" r:id="rId189"/>
-    <hyperlink ref="H191" r:id="rId190"/>
-    <hyperlink ref="H192" r:id="rId191"/>
-    <hyperlink ref="H193" r:id="rId192"/>
-    <hyperlink ref="H194" r:id="rId193"/>
-    <hyperlink ref="H195" r:id="rId194"/>
-    <hyperlink ref="H196" r:id="rId195"/>
-    <hyperlink ref="H197" r:id="rId196"/>
-    <hyperlink ref="H198" r:id="rId197"/>
-    <hyperlink ref="H199" r:id="rId198"/>
-    <hyperlink ref="H200" r:id="rId199"/>
-    <hyperlink ref="H201" r:id="rId200"/>
-    <hyperlink ref="H202" r:id="rId201"/>
-    <hyperlink ref="H203" r:id="rId202"/>
-    <hyperlink ref="H204" r:id="rId203"/>
-    <hyperlink ref="H205" r:id="rId204"/>
-    <hyperlink ref="H206" r:id="rId205"/>
-    <hyperlink ref="H207" r:id="rId206"/>
-    <hyperlink ref="H208" r:id="rId207"/>
-    <hyperlink ref="H209" r:id="rId208"/>
-    <hyperlink ref="H210" r:id="rId209"/>
-    <hyperlink ref="H211" r:id="rId210"/>
-    <hyperlink ref="H212" r:id="rId211"/>
-    <hyperlink ref="H213" r:id="rId212"/>
-    <hyperlink ref="H214" r:id="rId213"/>
-    <hyperlink ref="H215" r:id="rId214"/>
-    <hyperlink ref="H216" r:id="rId215"/>
-    <hyperlink ref="H217" r:id="rId216"/>
-    <hyperlink ref="H218" r:id="rId217"/>
-    <hyperlink ref="H219" r:id="rId218"/>
-    <hyperlink ref="H220" r:id="rId219"/>
-    <hyperlink ref="H221" r:id="rId220"/>
-    <hyperlink ref="H222" r:id="rId221"/>
-    <hyperlink ref="H223" r:id="rId222"/>
-    <hyperlink ref="H224" r:id="rId223"/>
-    <hyperlink ref="H225" r:id="rId224"/>
-    <hyperlink ref="H226" r:id="rId225"/>
-    <hyperlink ref="H227" r:id="rId226"/>
-    <hyperlink ref="H228" r:id="rId227"/>
-    <hyperlink ref="H229" r:id="rId228"/>
-    <hyperlink ref="H230" r:id="rId229"/>
-    <hyperlink ref="H231" r:id="rId230"/>
-    <hyperlink ref="H232" r:id="rId231"/>
-    <hyperlink ref="H233" r:id="rId232"/>
-    <hyperlink ref="H234" r:id="rId233"/>
-    <hyperlink ref="H235" r:id="rId234"/>
-    <hyperlink ref="H236" r:id="rId235"/>
-    <hyperlink ref="H237" r:id="rId236"/>
-    <hyperlink ref="H238" r:id="rId237"/>
-    <hyperlink ref="H239" r:id="rId238"/>
-    <hyperlink ref="H240" r:id="rId239"/>
-    <hyperlink ref="H241" r:id="rId240"/>
-    <hyperlink ref="H242" r:id="rId241"/>
-    <hyperlink ref="H243" r:id="rId242"/>
-    <hyperlink ref="H244" r:id="rId243"/>
-    <hyperlink ref="H245" r:id="rId244"/>
-    <hyperlink ref="H246" r:id="rId245"/>
-    <hyperlink ref="H247" r:id="rId246"/>
-    <hyperlink ref="H248" r:id="rId247"/>
-    <hyperlink ref="H249" r:id="rId248"/>
-    <hyperlink ref="H250" r:id="rId249"/>
-    <hyperlink ref="H251" r:id="rId250"/>
-    <hyperlink ref="H252" r:id="rId251"/>
-    <hyperlink ref="H253" r:id="rId252"/>
-    <hyperlink ref="H254" r:id="rId253"/>
-    <hyperlink ref="H255" r:id="rId254"/>
-    <hyperlink ref="H256" r:id="rId255"/>
-    <hyperlink ref="H257" r:id="rId256"/>
-    <hyperlink ref="H258" r:id="rId257"/>
-    <hyperlink ref="H259" r:id="rId258"/>
-    <hyperlink ref="H260" r:id="rId259"/>
-    <hyperlink ref="H261" r:id="rId260"/>
-    <hyperlink ref="H262" r:id="rId261"/>
-    <hyperlink ref="H263" r:id="rId262"/>
-    <hyperlink ref="H264" r:id="rId263"/>
-    <hyperlink ref="H265" r:id="rId264"/>
-    <hyperlink ref="H266" r:id="rId265"/>
-    <hyperlink ref="H267" r:id="rId266"/>
-    <hyperlink ref="H268" r:id="rId267"/>
-    <hyperlink ref="H269" r:id="rId268"/>
-    <hyperlink ref="H270" r:id="rId269"/>
-    <hyperlink ref="H271" r:id="rId270"/>
-    <hyperlink ref="H272" r:id="rId271"/>
-    <hyperlink ref="H273" r:id="rId272"/>
-    <hyperlink ref="H274" r:id="rId273"/>
-    <hyperlink ref="H275" r:id="rId274"/>
-    <hyperlink ref="H276" r:id="rId275"/>
-    <hyperlink ref="H277" r:id="rId276"/>
-    <hyperlink ref="H278" r:id="rId277"/>
-    <hyperlink ref="H279" r:id="rId278"/>
-    <hyperlink ref="H280" r:id="rId279"/>
-    <hyperlink ref="H281" r:id="rId280"/>
-    <hyperlink ref="H282" r:id="rId281"/>
-    <hyperlink ref="H283" r:id="rId282"/>
-    <hyperlink ref="H284" r:id="rId283"/>
-    <hyperlink ref="H285" r:id="rId284"/>
-    <hyperlink ref="H286" r:id="rId285"/>
-    <hyperlink ref="H287" r:id="rId286"/>
-    <hyperlink ref="H288" r:id="rId287"/>
-    <hyperlink ref="H289" r:id="rId288"/>
-    <hyperlink ref="H290" r:id="rId289"/>
-    <hyperlink ref="H291" r:id="rId290"/>
-    <hyperlink ref="H292" r:id="rId291"/>
-    <hyperlink ref="H293" r:id="rId292"/>
-    <hyperlink ref="H294" r:id="rId293"/>
-    <hyperlink ref="H295" r:id="rId294"/>
-    <hyperlink ref="H296" r:id="rId295"/>
-    <hyperlink ref="H297" r:id="rId296"/>
-    <hyperlink ref="H298" r:id="rId297"/>
-    <hyperlink ref="H299" r:id="rId298"/>
-    <hyperlink ref="H300" r:id="rId299"/>
-    <hyperlink ref="H301" r:id="rId300"/>
-    <hyperlink ref="H302" r:id="rId301"/>
-    <hyperlink ref="H303" r:id="rId302"/>
-    <hyperlink ref="H304" r:id="rId303"/>
-    <hyperlink ref="H305" r:id="rId304"/>
-    <hyperlink ref="H306" r:id="rId305"/>
-    <hyperlink ref="H307" r:id="rId306"/>
-    <hyperlink ref="H308" r:id="rId307"/>
-    <hyperlink ref="H309" r:id="rId308"/>
-    <hyperlink ref="H310" r:id="rId309"/>
-    <hyperlink ref="H311" r:id="rId310"/>
-    <hyperlink ref="H312" r:id="rId311"/>
-    <hyperlink ref="H313" r:id="rId312"/>
-    <hyperlink ref="H314" r:id="rId313"/>
-    <hyperlink ref="H315" r:id="rId314"/>
-    <hyperlink ref="H316" r:id="rId315"/>
-    <hyperlink ref="H317" r:id="rId316"/>
-    <hyperlink ref="H318" r:id="rId317"/>
-    <hyperlink ref="H319" r:id="rId318"/>
-    <hyperlink ref="H320" r:id="rId319"/>
-    <hyperlink ref="H321" r:id="rId320"/>
-    <hyperlink ref="H322" r:id="rId321"/>
-    <hyperlink ref="H323" r:id="rId322"/>
-    <hyperlink ref="H324" r:id="rId323"/>
-    <hyperlink ref="H325" r:id="rId324"/>
-    <hyperlink ref="H326" r:id="rId325"/>
-    <hyperlink ref="H327" r:id="rId326"/>
-    <hyperlink ref="H328" r:id="rId327"/>
-    <hyperlink ref="H329" r:id="rId328"/>
-    <hyperlink ref="H330" r:id="rId329"/>
-    <hyperlink ref="H331" r:id="rId330"/>
-    <hyperlink ref="H332" r:id="rId331"/>
-    <hyperlink ref="H333" r:id="rId332"/>
-    <hyperlink ref="H334" r:id="rId333"/>
-    <hyperlink ref="H335" r:id="rId334"/>
-    <hyperlink ref="H336" r:id="rId335"/>
-    <hyperlink ref="H337" r:id="rId336"/>
-    <hyperlink ref="H338" r:id="rId337"/>
-    <hyperlink ref="H339" r:id="rId338"/>
-    <hyperlink ref="H340" r:id="rId339"/>
-    <hyperlink ref="H341" r:id="rId340"/>
-    <hyperlink ref="H342" r:id="rId341"/>
-    <hyperlink ref="H343" r:id="rId342"/>
-    <hyperlink ref="H344" r:id="rId343"/>
-    <hyperlink ref="H345" r:id="rId344"/>
-    <hyperlink ref="H346" r:id="rId345"/>
-    <hyperlink ref="H347" r:id="rId346"/>
-    <hyperlink ref="H348" r:id="rId347"/>
-    <hyperlink ref="H349" r:id="rId348"/>
-    <hyperlink ref="H350" r:id="rId349"/>
-    <hyperlink ref="H351" r:id="rId350"/>
-    <hyperlink ref="H352" r:id="rId351"/>
-    <hyperlink ref="H353" r:id="rId352"/>
-    <hyperlink ref="H354" r:id="rId353"/>
-    <hyperlink ref="H355" r:id="rId354"/>
-    <hyperlink ref="H356" r:id="rId355"/>
-    <hyperlink ref="H357" r:id="rId356"/>
-    <hyperlink ref="H358" r:id="rId357"/>
-    <hyperlink ref="H359" r:id="rId358"/>
-    <hyperlink ref="H360" r:id="rId359"/>
-    <hyperlink ref="H361" r:id="rId360"/>
-    <hyperlink ref="H362" r:id="rId361"/>
-    <hyperlink ref="H363" r:id="rId362"/>
-    <hyperlink ref="H364" r:id="rId363"/>
-    <hyperlink ref="H365" r:id="rId364"/>
-    <hyperlink ref="H366" r:id="rId365"/>
-    <hyperlink ref="H367" r:id="rId366"/>
-    <hyperlink ref="H368" r:id="rId367"/>
-    <hyperlink ref="H369" r:id="rId368"/>
-    <hyperlink ref="H370" r:id="rId369"/>
-    <hyperlink ref="H371" r:id="rId370"/>
-    <hyperlink ref="H372" r:id="rId371"/>
-    <hyperlink ref="H373" r:id="rId372"/>
-    <hyperlink ref="H374" r:id="rId373"/>
-    <hyperlink ref="H375" r:id="rId374"/>
-    <hyperlink ref="H376" r:id="rId375"/>
-    <hyperlink ref="H377" r:id="rId376"/>
-    <hyperlink ref="H378" r:id="rId377"/>
-    <hyperlink ref="H379" r:id="rId378"/>
-    <hyperlink ref="H380" r:id="rId379"/>
-    <hyperlink ref="H381" r:id="rId380"/>
-    <hyperlink ref="H382" r:id="rId381"/>
-    <hyperlink ref="H383" r:id="rId382"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="H3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="H4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="H5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="H6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="H7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="H8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="H9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="H10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="H11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="H12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="H13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="H14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="H15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="H16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="H17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="H18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="H19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="H20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="H21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="H22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="H23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="H24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="H25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="H26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="H27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="H28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="H29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="H30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="H31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="H32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="H33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="H34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="H35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="H36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="H37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="H38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="H39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="H40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="H41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="H42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="H43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="H44" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="H45" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="H46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="H47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="H48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="H49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="H50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="H51" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="H52" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="H53" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="H54" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="H55" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="H56" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="H57" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="H58" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="H59" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="H60" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="H61" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="H62" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="H63" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="H64" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="H65" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="H66" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="H67" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="H68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="H69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="H70" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="H71" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="H72" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="H73" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="H74" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="H75" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="H76" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="H77" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="H78" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="H79" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="H80" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="H81" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="H82" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="H83" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="H84" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="H85" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="H86" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="H87" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="H88" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="H89" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="H90" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="H91" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="H92" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="H93" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="H94" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="H95" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="H96" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="H97" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="H98" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="H99" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="H100" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="H101" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="H102" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="H103" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="H104" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="H105" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="H106" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="H107" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="H108" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="H109" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="H110" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="H111" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="H112" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="H113" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="H114" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="H115" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="H116" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="H117" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="H118" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="H119" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="H120" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="H121" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
+    <hyperlink ref="H122" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
+    <hyperlink ref="H123" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
+    <hyperlink ref="H124" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="H125" r:id="rId124" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
+    <hyperlink ref="H126" r:id="rId125" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
+    <hyperlink ref="H127" r:id="rId126" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
+    <hyperlink ref="H128" r:id="rId127" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
+    <hyperlink ref="H129" r:id="rId128" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
+    <hyperlink ref="H130" r:id="rId129" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
+    <hyperlink ref="H131" r:id="rId130" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
+    <hyperlink ref="H132" r:id="rId131" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
+    <hyperlink ref="H133" r:id="rId132" xr:uid="{00000000-0004-0000-0000-000083000000}"/>
+    <hyperlink ref="H134" r:id="rId133" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
+    <hyperlink ref="H135" r:id="rId134" xr:uid="{00000000-0004-0000-0000-000085000000}"/>
+    <hyperlink ref="H136" r:id="rId135" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
+    <hyperlink ref="H137" r:id="rId136" xr:uid="{00000000-0004-0000-0000-000087000000}"/>
+    <hyperlink ref="H138" r:id="rId137" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
+    <hyperlink ref="H139" r:id="rId138" xr:uid="{00000000-0004-0000-0000-000089000000}"/>
+    <hyperlink ref="H140" r:id="rId139" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
+    <hyperlink ref="H141" r:id="rId140" xr:uid="{00000000-0004-0000-0000-00008B000000}"/>
+    <hyperlink ref="H142" r:id="rId141" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
+    <hyperlink ref="H143" r:id="rId142" xr:uid="{00000000-0004-0000-0000-00008D000000}"/>
+    <hyperlink ref="H144" r:id="rId143" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
+    <hyperlink ref="H145" r:id="rId144" xr:uid="{00000000-0004-0000-0000-00008F000000}"/>
+    <hyperlink ref="H146" r:id="rId145" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
+    <hyperlink ref="H147" r:id="rId146" xr:uid="{00000000-0004-0000-0000-000091000000}"/>
+    <hyperlink ref="H148" r:id="rId147" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
+    <hyperlink ref="H149" r:id="rId148" xr:uid="{00000000-0004-0000-0000-000093000000}"/>
+    <hyperlink ref="H150" r:id="rId149" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
+    <hyperlink ref="H151" r:id="rId150" xr:uid="{00000000-0004-0000-0000-000095000000}"/>
+    <hyperlink ref="H152" r:id="rId151" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
+    <hyperlink ref="H153" r:id="rId152" xr:uid="{00000000-0004-0000-0000-000097000000}"/>
+    <hyperlink ref="H154" r:id="rId153" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
+    <hyperlink ref="H155" r:id="rId154" xr:uid="{00000000-0004-0000-0000-000099000000}"/>
+    <hyperlink ref="H156" r:id="rId155" xr:uid="{00000000-0004-0000-0000-00009A000000}"/>
+    <hyperlink ref="H157" r:id="rId156" xr:uid="{00000000-0004-0000-0000-00009B000000}"/>
+    <hyperlink ref="H158" r:id="rId157" xr:uid="{00000000-0004-0000-0000-00009C000000}"/>
+    <hyperlink ref="H159" r:id="rId158" xr:uid="{00000000-0004-0000-0000-00009D000000}"/>
+    <hyperlink ref="H160" r:id="rId159" xr:uid="{00000000-0004-0000-0000-00009E000000}"/>
+    <hyperlink ref="H161" r:id="rId160" xr:uid="{00000000-0004-0000-0000-00009F000000}"/>
+    <hyperlink ref="H162" r:id="rId161" xr:uid="{00000000-0004-0000-0000-0000A0000000}"/>
+    <hyperlink ref="H163" r:id="rId162" xr:uid="{00000000-0004-0000-0000-0000A1000000}"/>
+    <hyperlink ref="H164" r:id="rId163" xr:uid="{00000000-0004-0000-0000-0000A2000000}"/>
+    <hyperlink ref="H165" r:id="rId164" xr:uid="{00000000-0004-0000-0000-0000A3000000}"/>
+    <hyperlink ref="H166" r:id="rId165" xr:uid="{00000000-0004-0000-0000-0000A4000000}"/>
+    <hyperlink ref="H167" r:id="rId166" xr:uid="{00000000-0004-0000-0000-0000A5000000}"/>
+    <hyperlink ref="H168" r:id="rId167" xr:uid="{00000000-0004-0000-0000-0000A6000000}"/>
+    <hyperlink ref="H169" r:id="rId168" xr:uid="{00000000-0004-0000-0000-0000A7000000}"/>
+    <hyperlink ref="H170" r:id="rId169" xr:uid="{00000000-0004-0000-0000-0000A8000000}"/>
+    <hyperlink ref="H171" r:id="rId170" xr:uid="{00000000-0004-0000-0000-0000A9000000}"/>
+    <hyperlink ref="H172" r:id="rId171" xr:uid="{00000000-0004-0000-0000-0000AA000000}"/>
+    <hyperlink ref="H173" r:id="rId172" xr:uid="{00000000-0004-0000-0000-0000AB000000}"/>
+    <hyperlink ref="H174" r:id="rId173" xr:uid="{00000000-0004-0000-0000-0000AC000000}"/>
+    <hyperlink ref="H175" r:id="rId174" xr:uid="{00000000-0004-0000-0000-0000AD000000}"/>
+    <hyperlink ref="H176" r:id="rId175" xr:uid="{00000000-0004-0000-0000-0000AE000000}"/>
+    <hyperlink ref="H177" r:id="rId176" xr:uid="{00000000-0004-0000-0000-0000AF000000}"/>
+    <hyperlink ref="H178" r:id="rId177" xr:uid="{00000000-0004-0000-0000-0000B0000000}"/>
+    <hyperlink ref="H179" r:id="rId178" xr:uid="{00000000-0004-0000-0000-0000B1000000}"/>
+    <hyperlink ref="H180" r:id="rId179" xr:uid="{00000000-0004-0000-0000-0000B2000000}"/>
+    <hyperlink ref="H181" r:id="rId180" xr:uid="{00000000-0004-0000-0000-0000B3000000}"/>
+    <hyperlink ref="H182" r:id="rId181" xr:uid="{00000000-0004-0000-0000-0000B4000000}"/>
+    <hyperlink ref="H183" r:id="rId182" xr:uid="{00000000-0004-0000-0000-0000B5000000}"/>
+    <hyperlink ref="H184" r:id="rId183" xr:uid="{00000000-0004-0000-0000-0000B6000000}"/>
+    <hyperlink ref="H185" r:id="rId184" xr:uid="{00000000-0004-0000-0000-0000B7000000}"/>
+    <hyperlink ref="H186" r:id="rId185" xr:uid="{00000000-0004-0000-0000-0000B8000000}"/>
+    <hyperlink ref="H187" r:id="rId186" xr:uid="{00000000-0004-0000-0000-0000B9000000}"/>
+    <hyperlink ref="H188" r:id="rId187" xr:uid="{00000000-0004-0000-0000-0000BA000000}"/>
+    <hyperlink ref="H189" r:id="rId188" xr:uid="{00000000-0004-0000-0000-0000BB000000}"/>
+    <hyperlink ref="H190" r:id="rId189" xr:uid="{00000000-0004-0000-0000-0000BC000000}"/>
+    <hyperlink ref="H191" r:id="rId190" xr:uid="{00000000-0004-0000-0000-0000BD000000}"/>
+    <hyperlink ref="H192" r:id="rId191" xr:uid="{00000000-0004-0000-0000-0000BE000000}"/>
+    <hyperlink ref="H193" r:id="rId192" xr:uid="{00000000-0004-0000-0000-0000BF000000}"/>
+    <hyperlink ref="H194" r:id="rId193" xr:uid="{00000000-0004-0000-0000-0000C0000000}"/>
+    <hyperlink ref="H195" r:id="rId194" xr:uid="{00000000-0004-0000-0000-0000C1000000}"/>
+    <hyperlink ref="H196" r:id="rId195" xr:uid="{00000000-0004-0000-0000-0000C2000000}"/>
+    <hyperlink ref="H197" r:id="rId196" xr:uid="{00000000-0004-0000-0000-0000C3000000}"/>
+    <hyperlink ref="H198" r:id="rId197" xr:uid="{00000000-0004-0000-0000-0000C4000000}"/>
+    <hyperlink ref="H199" r:id="rId198" xr:uid="{00000000-0004-0000-0000-0000C5000000}"/>
+    <hyperlink ref="H200" r:id="rId199" xr:uid="{00000000-0004-0000-0000-0000C6000000}"/>
+    <hyperlink ref="H201" r:id="rId200" xr:uid="{00000000-0004-0000-0000-0000C7000000}"/>
+    <hyperlink ref="H202" r:id="rId201" xr:uid="{00000000-0004-0000-0000-0000C8000000}"/>
+    <hyperlink ref="H203" r:id="rId202" xr:uid="{00000000-0004-0000-0000-0000C9000000}"/>
+    <hyperlink ref="H204" r:id="rId203" xr:uid="{00000000-0004-0000-0000-0000CA000000}"/>
+    <hyperlink ref="H205" r:id="rId204" xr:uid="{00000000-0004-0000-0000-0000CB000000}"/>
+    <hyperlink ref="H206" r:id="rId205" xr:uid="{00000000-0004-0000-0000-0000CC000000}"/>
+    <hyperlink ref="H207" r:id="rId206" xr:uid="{00000000-0004-0000-0000-0000CD000000}"/>
+    <hyperlink ref="H208" r:id="rId207" xr:uid="{00000000-0004-0000-0000-0000CE000000}"/>
+    <hyperlink ref="H209" r:id="rId208" xr:uid="{00000000-0004-0000-0000-0000CF000000}"/>
+    <hyperlink ref="H210" r:id="rId209" xr:uid="{00000000-0004-0000-0000-0000D0000000}"/>
+    <hyperlink ref="H211" r:id="rId210" xr:uid="{00000000-0004-0000-0000-0000D1000000}"/>
+    <hyperlink ref="H212" r:id="rId211" xr:uid="{00000000-0004-0000-0000-0000D2000000}"/>
+    <hyperlink ref="H213" r:id="rId212" xr:uid="{00000000-0004-0000-0000-0000D3000000}"/>
+    <hyperlink ref="H214" r:id="rId213" xr:uid="{00000000-0004-0000-0000-0000D4000000}"/>
+    <hyperlink ref="H215" r:id="rId214" xr:uid="{00000000-0004-0000-0000-0000D5000000}"/>
+    <hyperlink ref="H216" r:id="rId215" xr:uid="{00000000-0004-0000-0000-0000D6000000}"/>
+    <hyperlink ref="H217" r:id="rId216" xr:uid="{00000000-0004-0000-0000-0000D7000000}"/>
+    <hyperlink ref="H218" r:id="rId217" xr:uid="{00000000-0004-0000-0000-0000D8000000}"/>
+    <hyperlink ref="H219" r:id="rId218" xr:uid="{00000000-0004-0000-0000-0000D9000000}"/>
+    <hyperlink ref="H220" r:id="rId219" xr:uid="{00000000-0004-0000-0000-0000DA000000}"/>
+    <hyperlink ref="H221" r:id="rId220" xr:uid="{00000000-0004-0000-0000-0000DB000000}"/>
+    <hyperlink ref="H222" r:id="rId221" xr:uid="{00000000-0004-0000-0000-0000DC000000}"/>
+    <hyperlink ref="H223" r:id="rId222" xr:uid="{00000000-0004-0000-0000-0000DD000000}"/>
+    <hyperlink ref="H224" r:id="rId223" xr:uid="{00000000-0004-0000-0000-0000DE000000}"/>
+    <hyperlink ref="H225" r:id="rId224" xr:uid="{00000000-0004-0000-0000-0000DF000000}"/>
+    <hyperlink ref="H226" r:id="rId225" xr:uid="{00000000-0004-0000-0000-0000E0000000}"/>
+    <hyperlink ref="H227" r:id="rId226" xr:uid="{00000000-0004-0000-0000-0000E1000000}"/>
+    <hyperlink ref="H228" r:id="rId227" xr:uid="{00000000-0004-0000-0000-0000E2000000}"/>
+    <hyperlink ref="H229" r:id="rId228" xr:uid="{00000000-0004-0000-0000-0000E3000000}"/>
+    <hyperlink ref="H230" r:id="rId229" xr:uid="{00000000-0004-0000-0000-0000E4000000}"/>
+    <hyperlink ref="H231" r:id="rId230" xr:uid="{00000000-0004-0000-0000-0000E5000000}"/>
+    <hyperlink ref="H232" r:id="rId231" xr:uid="{00000000-0004-0000-0000-0000E6000000}"/>
+    <hyperlink ref="H233" r:id="rId232" xr:uid="{00000000-0004-0000-0000-0000E7000000}"/>
+    <hyperlink ref="H234" r:id="rId233" xr:uid="{00000000-0004-0000-0000-0000E8000000}"/>
+    <hyperlink ref="H235" r:id="rId234" xr:uid="{00000000-0004-0000-0000-0000E9000000}"/>
+    <hyperlink ref="H236" r:id="rId235" xr:uid="{00000000-0004-0000-0000-0000EA000000}"/>
+    <hyperlink ref="H237" r:id="rId236" xr:uid="{00000000-0004-0000-0000-0000EB000000}"/>
+    <hyperlink ref="H238" r:id="rId237" xr:uid="{00000000-0004-0000-0000-0000EC000000}"/>
+    <hyperlink ref="H239" r:id="rId238" xr:uid="{00000000-0004-0000-0000-0000ED000000}"/>
+    <hyperlink ref="H240" r:id="rId239" xr:uid="{00000000-0004-0000-0000-0000EE000000}"/>
+    <hyperlink ref="H241" r:id="rId240" xr:uid="{00000000-0004-0000-0000-0000EF000000}"/>
+    <hyperlink ref="H242" r:id="rId241" xr:uid="{00000000-0004-0000-0000-0000F0000000}"/>
+    <hyperlink ref="H243" r:id="rId242" xr:uid="{00000000-0004-0000-0000-0000F1000000}"/>
+    <hyperlink ref="H244" r:id="rId243" xr:uid="{00000000-0004-0000-0000-0000F2000000}"/>
+    <hyperlink ref="H245" r:id="rId244" xr:uid="{00000000-0004-0000-0000-0000F3000000}"/>
+    <hyperlink ref="H246" r:id="rId245" xr:uid="{00000000-0004-0000-0000-0000F4000000}"/>
+    <hyperlink ref="H247" r:id="rId246" xr:uid="{00000000-0004-0000-0000-0000F5000000}"/>
+    <hyperlink ref="H248" r:id="rId247" xr:uid="{00000000-0004-0000-0000-0000F6000000}"/>
+    <hyperlink ref="H249" r:id="rId248" xr:uid="{00000000-0004-0000-0000-0000F7000000}"/>
+    <hyperlink ref="H250" r:id="rId249" xr:uid="{00000000-0004-0000-0000-0000F8000000}"/>
+    <hyperlink ref="H251" r:id="rId250" xr:uid="{00000000-0004-0000-0000-0000F9000000}"/>
+    <hyperlink ref="H252" r:id="rId251" xr:uid="{00000000-0004-0000-0000-0000FA000000}"/>
+    <hyperlink ref="H253" r:id="rId252" xr:uid="{00000000-0004-0000-0000-0000FB000000}"/>
+    <hyperlink ref="H254" r:id="rId253" xr:uid="{00000000-0004-0000-0000-0000FC000000}"/>
+    <hyperlink ref="H255" r:id="rId254" xr:uid="{00000000-0004-0000-0000-0000FD000000}"/>
+    <hyperlink ref="H256" r:id="rId255" xr:uid="{00000000-0004-0000-0000-0000FE000000}"/>
+    <hyperlink ref="H257" r:id="rId256" xr:uid="{00000000-0004-0000-0000-0000FF000000}"/>
+    <hyperlink ref="H258" r:id="rId257" xr:uid="{00000000-0004-0000-0000-000000010000}"/>
+    <hyperlink ref="H259" r:id="rId258" xr:uid="{00000000-0004-0000-0000-000001010000}"/>
+    <hyperlink ref="H260" r:id="rId259" xr:uid="{00000000-0004-0000-0000-000002010000}"/>
+    <hyperlink ref="H261" r:id="rId260" xr:uid="{00000000-0004-0000-0000-000003010000}"/>
+    <hyperlink ref="H262" r:id="rId261" xr:uid="{00000000-0004-0000-0000-000004010000}"/>
+    <hyperlink ref="H263" r:id="rId262" xr:uid="{00000000-0004-0000-0000-000005010000}"/>
+    <hyperlink ref="H264" r:id="rId263" xr:uid="{00000000-0004-0000-0000-000006010000}"/>
+    <hyperlink ref="H265" r:id="rId264" xr:uid="{00000000-0004-0000-0000-000007010000}"/>
+    <hyperlink ref="H266" r:id="rId265" xr:uid="{00000000-0004-0000-0000-000008010000}"/>
+    <hyperlink ref="H267" r:id="rId266" xr:uid="{00000000-0004-0000-0000-000009010000}"/>
+    <hyperlink ref="H268" r:id="rId267" xr:uid="{00000000-0004-0000-0000-00000A010000}"/>
+    <hyperlink ref="H269" r:id="rId268" xr:uid="{00000000-0004-0000-0000-00000B010000}"/>
+    <hyperlink ref="H270" r:id="rId269" xr:uid="{00000000-0004-0000-0000-00000C010000}"/>
+    <hyperlink ref="H271" r:id="rId270" xr:uid="{00000000-0004-0000-0000-00000D010000}"/>
+    <hyperlink ref="H272" r:id="rId271" xr:uid="{00000000-0004-0000-0000-00000E010000}"/>
+    <hyperlink ref="H273" r:id="rId272" xr:uid="{00000000-0004-0000-0000-00000F010000}"/>
+    <hyperlink ref="H274" r:id="rId273" xr:uid="{00000000-0004-0000-0000-000010010000}"/>
+    <hyperlink ref="H275" r:id="rId274" xr:uid="{00000000-0004-0000-0000-000011010000}"/>
+    <hyperlink ref="H276" r:id="rId275" xr:uid="{00000000-0004-0000-0000-000012010000}"/>
+    <hyperlink ref="H277" r:id="rId276" xr:uid="{00000000-0004-0000-0000-000013010000}"/>
+    <hyperlink ref="H278" r:id="rId277" xr:uid="{00000000-0004-0000-0000-000014010000}"/>
+    <hyperlink ref="H279" r:id="rId278" xr:uid="{00000000-0004-0000-0000-000015010000}"/>
+    <hyperlink ref="H280" r:id="rId279" xr:uid="{00000000-0004-0000-0000-000016010000}"/>
+    <hyperlink ref="H281" r:id="rId280" xr:uid="{00000000-0004-0000-0000-000017010000}"/>
+    <hyperlink ref="H282" r:id="rId281" xr:uid="{00000000-0004-0000-0000-000018010000}"/>
+    <hyperlink ref="H283" r:id="rId282" xr:uid="{00000000-0004-0000-0000-000019010000}"/>
+    <hyperlink ref="H284" r:id="rId283" xr:uid="{00000000-0004-0000-0000-00001A010000}"/>
+    <hyperlink ref="H285" r:id="rId284" xr:uid="{00000000-0004-0000-0000-00001B010000}"/>
+    <hyperlink ref="H286" r:id="rId285" xr:uid="{00000000-0004-0000-0000-00001C010000}"/>
+    <hyperlink ref="H287" r:id="rId286" xr:uid="{00000000-0004-0000-0000-00001D010000}"/>
+    <hyperlink ref="H288" r:id="rId287" xr:uid="{00000000-0004-0000-0000-00001E010000}"/>
+    <hyperlink ref="H289" r:id="rId288" xr:uid="{00000000-0004-0000-0000-00001F010000}"/>
+    <hyperlink ref="H290" r:id="rId289" xr:uid="{00000000-0004-0000-0000-000020010000}"/>
+    <hyperlink ref="H291" r:id="rId290" xr:uid="{00000000-0004-0000-0000-000021010000}"/>
+    <hyperlink ref="H292" r:id="rId291" xr:uid="{00000000-0004-0000-0000-000022010000}"/>
+    <hyperlink ref="H293" r:id="rId292" xr:uid="{00000000-0004-0000-0000-000023010000}"/>
+    <hyperlink ref="H294" r:id="rId293" xr:uid="{00000000-0004-0000-0000-000024010000}"/>
+    <hyperlink ref="H295" r:id="rId294" xr:uid="{00000000-0004-0000-0000-000025010000}"/>
+    <hyperlink ref="H296" r:id="rId295" xr:uid="{00000000-0004-0000-0000-000026010000}"/>
+    <hyperlink ref="H297" r:id="rId296" xr:uid="{00000000-0004-0000-0000-000027010000}"/>
+    <hyperlink ref="H298" r:id="rId297" xr:uid="{00000000-0004-0000-0000-000028010000}"/>
+    <hyperlink ref="H299" r:id="rId298" xr:uid="{00000000-0004-0000-0000-000029010000}"/>
+    <hyperlink ref="H300" r:id="rId299" xr:uid="{00000000-0004-0000-0000-00002A010000}"/>
+    <hyperlink ref="H301" r:id="rId300" xr:uid="{00000000-0004-0000-0000-00002B010000}"/>
+    <hyperlink ref="H302" r:id="rId301" xr:uid="{00000000-0004-0000-0000-00002C010000}"/>
+    <hyperlink ref="H303" r:id="rId302" xr:uid="{00000000-0004-0000-0000-00002D010000}"/>
+    <hyperlink ref="H304" r:id="rId303" xr:uid="{00000000-0004-0000-0000-00002E010000}"/>
+    <hyperlink ref="H305" r:id="rId304" xr:uid="{00000000-0004-0000-0000-00002F010000}"/>
+    <hyperlink ref="H306" r:id="rId305" xr:uid="{00000000-0004-0000-0000-000030010000}"/>
+    <hyperlink ref="H307" r:id="rId306" xr:uid="{00000000-0004-0000-0000-000031010000}"/>
+    <hyperlink ref="H308" r:id="rId307" xr:uid="{00000000-0004-0000-0000-000032010000}"/>
+    <hyperlink ref="H309" r:id="rId308" xr:uid="{00000000-0004-0000-0000-000033010000}"/>
+    <hyperlink ref="H310" r:id="rId309" xr:uid="{00000000-0004-0000-0000-000034010000}"/>
+    <hyperlink ref="H311" r:id="rId310" xr:uid="{00000000-0004-0000-0000-000035010000}"/>
+    <hyperlink ref="H312" r:id="rId311" xr:uid="{00000000-0004-0000-0000-000036010000}"/>
+    <hyperlink ref="H313" r:id="rId312" xr:uid="{00000000-0004-0000-0000-000037010000}"/>
+    <hyperlink ref="H314" r:id="rId313" xr:uid="{00000000-0004-0000-0000-000038010000}"/>
+    <hyperlink ref="H315" r:id="rId314" xr:uid="{00000000-0004-0000-0000-000039010000}"/>
+    <hyperlink ref="H316" r:id="rId315" xr:uid="{00000000-0004-0000-0000-00003A010000}"/>
+    <hyperlink ref="H317" r:id="rId316" xr:uid="{00000000-0004-0000-0000-00003B010000}"/>
+    <hyperlink ref="H318" r:id="rId317" xr:uid="{00000000-0004-0000-0000-00003C010000}"/>
+    <hyperlink ref="H319" r:id="rId318" xr:uid="{00000000-0004-0000-0000-00003D010000}"/>
+    <hyperlink ref="H320" r:id="rId319" xr:uid="{00000000-0004-0000-0000-00003E010000}"/>
+    <hyperlink ref="H321" r:id="rId320" xr:uid="{00000000-0004-0000-0000-00003F010000}"/>
+    <hyperlink ref="H322" r:id="rId321" xr:uid="{00000000-0004-0000-0000-000040010000}"/>
+    <hyperlink ref="H323" r:id="rId322" xr:uid="{00000000-0004-0000-0000-000041010000}"/>
+    <hyperlink ref="H324" r:id="rId323" xr:uid="{00000000-0004-0000-0000-000042010000}"/>
+    <hyperlink ref="H325" r:id="rId324" xr:uid="{00000000-0004-0000-0000-000043010000}"/>
+    <hyperlink ref="H326" r:id="rId325" xr:uid="{00000000-0004-0000-0000-000044010000}"/>
+    <hyperlink ref="H327" r:id="rId326" xr:uid="{00000000-0004-0000-0000-000045010000}"/>
+    <hyperlink ref="H328" r:id="rId327" xr:uid="{00000000-0004-0000-0000-000046010000}"/>
+    <hyperlink ref="H329" r:id="rId328" xr:uid="{00000000-0004-0000-0000-000047010000}"/>
+    <hyperlink ref="H330" r:id="rId329" xr:uid="{00000000-0004-0000-0000-000048010000}"/>
+    <hyperlink ref="H331" r:id="rId330" xr:uid="{00000000-0004-0000-0000-000049010000}"/>
+    <hyperlink ref="H332" r:id="rId331" xr:uid="{00000000-0004-0000-0000-00004A010000}"/>
+    <hyperlink ref="H333" r:id="rId332" xr:uid="{00000000-0004-0000-0000-00004B010000}"/>
+    <hyperlink ref="H334" r:id="rId333" xr:uid="{00000000-0004-0000-0000-00004C010000}"/>
+    <hyperlink ref="H335" r:id="rId334" xr:uid="{00000000-0004-0000-0000-00004D010000}"/>
+    <hyperlink ref="H336" r:id="rId335" xr:uid="{00000000-0004-0000-0000-00004E010000}"/>
+    <hyperlink ref="H337" r:id="rId336" xr:uid="{00000000-0004-0000-0000-00004F010000}"/>
+    <hyperlink ref="H338" r:id="rId337" xr:uid="{00000000-0004-0000-0000-000050010000}"/>
+    <hyperlink ref="H339" r:id="rId338" xr:uid="{00000000-0004-0000-0000-000051010000}"/>
+    <hyperlink ref="H340" r:id="rId339" xr:uid="{00000000-0004-0000-0000-000052010000}"/>
+    <hyperlink ref="H341" r:id="rId340" xr:uid="{00000000-0004-0000-0000-000053010000}"/>
+    <hyperlink ref="H342" r:id="rId341" xr:uid="{00000000-0004-0000-0000-000054010000}"/>
+    <hyperlink ref="H343" r:id="rId342" xr:uid="{00000000-0004-0000-0000-000055010000}"/>
+    <hyperlink ref="H344" r:id="rId343" xr:uid="{00000000-0004-0000-0000-000056010000}"/>
+    <hyperlink ref="H345" r:id="rId344" xr:uid="{00000000-0004-0000-0000-000057010000}"/>
+    <hyperlink ref="H346" r:id="rId345" xr:uid="{00000000-0004-0000-0000-000058010000}"/>
+    <hyperlink ref="H347" r:id="rId346" xr:uid="{00000000-0004-0000-0000-000059010000}"/>
+    <hyperlink ref="H348" r:id="rId347" xr:uid="{00000000-0004-0000-0000-00005A010000}"/>
+    <hyperlink ref="H349" r:id="rId348" xr:uid="{00000000-0004-0000-0000-00005B010000}"/>
+    <hyperlink ref="H350" r:id="rId349" xr:uid="{00000000-0004-0000-0000-00005C010000}"/>
+    <hyperlink ref="H351" r:id="rId350" xr:uid="{00000000-0004-0000-0000-00005D010000}"/>
+    <hyperlink ref="H352" r:id="rId351" xr:uid="{00000000-0004-0000-0000-00005E010000}"/>
+    <hyperlink ref="H353" r:id="rId352" xr:uid="{00000000-0004-0000-0000-00005F010000}"/>
+    <hyperlink ref="H354" r:id="rId353" xr:uid="{00000000-0004-0000-0000-000060010000}"/>
+    <hyperlink ref="H355" r:id="rId354" xr:uid="{00000000-0004-0000-0000-000061010000}"/>
+    <hyperlink ref="H356" r:id="rId355" xr:uid="{00000000-0004-0000-0000-000062010000}"/>
+    <hyperlink ref="H357" r:id="rId356" xr:uid="{00000000-0004-0000-0000-000063010000}"/>
+    <hyperlink ref="H358" r:id="rId357" xr:uid="{00000000-0004-0000-0000-000064010000}"/>
+    <hyperlink ref="H359" r:id="rId358" xr:uid="{00000000-0004-0000-0000-000065010000}"/>
+    <hyperlink ref="H360" r:id="rId359" xr:uid="{00000000-0004-0000-0000-000066010000}"/>
+    <hyperlink ref="H361" r:id="rId360" xr:uid="{00000000-0004-0000-0000-000067010000}"/>
+    <hyperlink ref="H362" r:id="rId361" xr:uid="{00000000-0004-0000-0000-000068010000}"/>
+    <hyperlink ref="H363" r:id="rId362" xr:uid="{00000000-0004-0000-0000-000069010000}"/>
+    <hyperlink ref="H364" r:id="rId363" xr:uid="{00000000-0004-0000-0000-00006A010000}"/>
+    <hyperlink ref="H365" r:id="rId364" xr:uid="{00000000-0004-0000-0000-00006B010000}"/>
+    <hyperlink ref="H366" r:id="rId365" xr:uid="{00000000-0004-0000-0000-00006C010000}"/>
+    <hyperlink ref="H367" r:id="rId366" xr:uid="{00000000-0004-0000-0000-00006D010000}"/>
+    <hyperlink ref="H368" r:id="rId367" xr:uid="{00000000-0004-0000-0000-00006E010000}"/>
+    <hyperlink ref="H369" r:id="rId368" xr:uid="{00000000-0004-0000-0000-00006F010000}"/>
+    <hyperlink ref="H370" r:id="rId369" xr:uid="{00000000-0004-0000-0000-000070010000}"/>
+    <hyperlink ref="H371" r:id="rId370" xr:uid="{00000000-0004-0000-0000-000071010000}"/>
+    <hyperlink ref="H372" r:id="rId371" xr:uid="{00000000-0004-0000-0000-000072010000}"/>
+    <hyperlink ref="H373" r:id="rId372" xr:uid="{00000000-0004-0000-0000-000073010000}"/>
+    <hyperlink ref="H374" r:id="rId373" xr:uid="{00000000-0004-0000-0000-000074010000}"/>
+    <hyperlink ref="H375" r:id="rId374" xr:uid="{00000000-0004-0000-0000-000075010000}"/>
+    <hyperlink ref="H376" r:id="rId375" xr:uid="{00000000-0004-0000-0000-000076010000}"/>
+    <hyperlink ref="H377" r:id="rId376" xr:uid="{00000000-0004-0000-0000-000077010000}"/>
+    <hyperlink ref="H378" r:id="rId377" xr:uid="{00000000-0004-0000-0000-000078010000}"/>
+    <hyperlink ref="H379" r:id="rId378" xr:uid="{00000000-0004-0000-0000-000079010000}"/>
+    <hyperlink ref="H380" r:id="rId379" xr:uid="{00000000-0004-0000-0000-00007A010000}"/>
+    <hyperlink ref="H381" r:id="rId380" xr:uid="{00000000-0004-0000-0000-00007B010000}"/>
+    <hyperlink ref="H382" r:id="rId381" xr:uid="{00000000-0004-0000-0000-00007C010000}"/>
+    <hyperlink ref="H383" r:id="rId382" xr:uid="{00000000-0004-0000-0000-00007D010000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52CC5AF5-E264-49D1-86F6-D467FA16355B}">
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="39" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>756</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>757</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>759</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>761</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>763</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>765</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>767</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>769</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>777</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>779</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>785</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>787</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>789</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>791</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>794</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{C551F7C9-B5B4-4F31-81A7-A83B9C6E9DA5}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{295C38C1-0317-457A-9A3D-50B4F19D8269}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{F8EA3C10-CDA1-4F5F-BA61-4954037E4B1E}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{7217B163-A17D-4B95-B96D-EDA896C1C4D0}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{CAF67487-DD44-4BA6-B680-80DB007897BB}"/>
+    <hyperlink ref="C7" r:id="rId6" xr:uid="{5C776465-7753-47C3-90EA-27F8A47111C4}"/>
+    <hyperlink ref="C8" r:id="rId7" xr:uid="{FD425C97-1F53-4515-B65D-7C292A2A0044}"/>
+    <hyperlink ref="C9" r:id="rId8" xr:uid="{92A45463-3EA6-4047-8586-AC267584B69E}"/>
+    <hyperlink ref="C10" r:id="rId9" xr:uid="{2871430C-2D48-48C9-B950-E7DAC23D7D4C}"/>
+    <hyperlink ref="C11" r:id="rId10" xr:uid="{857C0888-9FED-4039-AF51-90CB93443DED}"/>
+    <hyperlink ref="C12" r:id="rId11" xr:uid="{DA9B8B37-F610-438D-B6CA-A8D014C01214}"/>
+    <hyperlink ref="C13" r:id="rId12" xr:uid="{A37FB7F3-7CF9-41BD-902E-AC79C21496BB}"/>
+    <hyperlink ref="C14" r:id="rId13" xr:uid="{833BC2EF-1BEE-4249-B345-F3280117FF9D}"/>
+    <hyperlink ref="C15" r:id="rId14" xr:uid="{579E5158-3B8D-4937-9B45-AB08D07BB71E}"/>
+    <hyperlink ref="C16" r:id="rId15" xr:uid="{8EB18D6A-FDA5-4995-BF35-47D4FEAFE9D3}"/>
+    <hyperlink ref="C17" r:id="rId16" xr:uid="{88551A69-B711-4C0A-9143-DC354E082D57}"/>
+    <hyperlink ref="C18" r:id="rId17" xr:uid="{69A0799F-0120-48C8-9B80-E63EC84B0E8B}"/>
+    <hyperlink ref="C19" r:id="rId18" xr:uid="{92CB2047-DBE8-4D7C-9572-679ABB9029FA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>